<commit_message>
updated list and animation
</commit_message>
<xml_diff>
--- a/brown_signs.xlsx
+++ b/brown_signs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ozbek\Desktop\brown_signs_denmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC25C97-4AF9-45F2-A2D1-8AB8DC555FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92BF5A5C-6AB2-47F6-9456-6CD86216AF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{1A3F83CA-556E-4C31-A6BA-F78F2B7B4EED}"/>
   </bookViews>
@@ -939,10 +939,10 @@
         <v>68</v>
       </c>
       <c r="B6">
-        <v>57.34</v>
+        <v>57.3691547377083</v>
       </c>
       <c r="C6">
-        <v>9.77</v>
+        <v>9.7994446959873205</v>
       </c>
       <c r="D6">
         <v>57.3584673055108</v>
@@ -959,10 +959,10 @@
         <v>64</v>
       </c>
       <c r="B7">
-        <v>57.174999999999997</v>
+        <v>57.242624856684898</v>
       </c>
       <c r="C7">
-        <v>10.27</v>
+        <v>10.336018084347399</v>
       </c>
       <c r="D7">
         <v>57.2470180636668</v>
@@ -979,10 +979,10 @@
         <v>70</v>
       </c>
       <c r="B8">
-        <v>57.146999999999998</v>
+        <v>57.270661191574398</v>
       </c>
       <c r="C8">
-        <v>9.69</v>
+        <v>9.6500354727138298</v>
       </c>
       <c r="D8">
         <v>57.197781406415899</v>
@@ -999,10 +999,10 @@
         <v>65</v>
       </c>
       <c r="B9">
-        <v>57.14</v>
+        <v>57.167811312996001</v>
       </c>
       <c r="C9">
-        <v>10.32</v>
+        <v>10.258205848085201</v>
       </c>
       <c r="D9">
         <v>57.165319955585197</v>
@@ -1019,10 +1019,10 @@
         <v>69</v>
       </c>
       <c r="B10">
-        <v>57.1</v>
+        <v>57.208603588639797</v>
       </c>
       <c r="C10">
-        <v>9.77</v>
+        <v>9.8098167757515196</v>
       </c>
       <c r="D10">
         <v>57.247566866366803</v>
@@ -1039,10 +1039,10 @@
         <v>2</v>
       </c>
       <c r="B11">
-        <v>57.061999999999998</v>
+        <v>57.0777324845062</v>
       </c>
       <c r="C11">
-        <v>9.9139999999999997</v>
+        <v>9.9124300989358805</v>
       </c>
       <c r="D11">
         <v>57.067395297684001</v>
@@ -1059,10 +1059,10 @@
         <v>3</v>
       </c>
       <c r="B12">
-        <v>57.042499999999997</v>
+        <v>57.0426823598089</v>
       </c>
       <c r="C12">
-        <v>9.9130000000000003</v>
+        <v>9.9063698131759104</v>
       </c>
       <c r="D12">
         <v>57.030231552493099</v>
@@ -1079,10 +1079,10 @@
         <v>4</v>
       </c>
       <c r="B13">
-        <v>57.04</v>
+        <v>57.037146523820503</v>
       </c>
       <c r="C13">
-        <v>9.8970000000000002</v>
+        <v>9.89855878248345</v>
       </c>
       <c r="D13">
         <v>57.001754305740398</v>
@@ -1119,10 +1119,10 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>56.884999999999998</v>
+        <v>56.884710494084999</v>
       </c>
       <c r="C15">
-        <v>10.220000000000001</v>
+        <v>10.194378444915801</v>
       </c>
       <c r="D15">
         <v>56.9532637837411</v>
@@ -1139,10 +1139,10 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>56.837000000000003</v>
+        <v>56.831372000743599</v>
       </c>
       <c r="C16">
-        <v>9.84</v>
+        <v>9.8432852447139201</v>
       </c>
       <c r="D16">
         <v>56.877442007742999</v>
@@ -1159,10 +1159,10 @@
         <v>7</v>
       </c>
       <c r="B17">
-        <v>56.804000000000002</v>
+        <v>56.800965374106497</v>
       </c>
       <c r="C17">
-        <v>9.5180000000000007</v>
+        <v>9.5297844005768493</v>
       </c>
       <c r="D17">
         <v>56.831024640751203</v>
@@ -1179,10 +1179,10 @@
         <v>8</v>
       </c>
       <c r="B18">
-        <v>56.78</v>
+        <v>56.799532874083397</v>
       </c>
       <c r="C18">
-        <v>9.94</v>
+        <v>9.8217308890124002</v>
       </c>
       <c r="D18">
         <v>56.786739778388899</v>
@@ -1199,10 +1199,10 @@
         <v>11</v>
       </c>
       <c r="B19">
-        <v>56.643000000000001</v>
+        <v>56.650024928667797</v>
       </c>
       <c r="C19">
-        <v>10.023999999999999</v>
+        <v>9.9772687538191391</v>
       </c>
       <c r="D19">
         <v>56.579258536130503</v>
@@ -1219,10 +1219,10 @@
         <v>9</v>
       </c>
       <c r="B20">
-        <v>56.634999999999998</v>
+        <v>56.625065922939399</v>
       </c>
       <c r="C20">
-        <v>9.7899999999999991</v>
+        <v>9.7724621619073506</v>
       </c>
       <c r="D20">
         <v>56.622353820633201</v>
@@ -1239,10 +1239,10 @@
         <v>10</v>
       </c>
       <c r="B21">
-        <v>56.551000000000002</v>
+        <v>56.590573153528901</v>
       </c>
       <c r="C21">
-        <v>9.5489999999999995</v>
+        <v>9.6409248902011093</v>
       </c>
       <c r="D21">
         <v>56.588378787362998</v>
@@ -1259,10 +1259,10 @@
         <v>12</v>
       </c>
       <c r="B22">
-        <v>56.54</v>
+        <v>56.556176738759902</v>
       </c>
       <c r="C22">
-        <v>9.84</v>
+        <v>10.0025354539068</v>
       </c>
       <c r="D22">
         <v>56.540406347137903</v>
@@ -1279,10 +1279,10 @@
         <v>80</v>
       </c>
       <c r="B23">
-        <v>56.466999999999999</v>
+        <v>56.484518202766601</v>
       </c>
       <c r="C23">
-        <v>8.7989999999999995</v>
+        <v>8.8695367959516904</v>
       </c>
       <c r="D23">
         <v>56.363541782240297</v>
@@ -1299,10 +1299,10 @@
         <v>13</v>
       </c>
       <c r="B24">
-        <v>56.462000000000003</v>
+        <v>56.460499790466102</v>
       </c>
       <c r="C24">
-        <v>10.038</v>
+        <v>10.041525732209999</v>
       </c>
       <c r="D24">
         <v>56.486205569362397</v>
@@ -1319,10 +1319,10 @@
         <v>14</v>
       </c>
       <c r="B25">
-        <v>56.462000000000003</v>
+        <v>56.457271281324999</v>
       </c>
       <c r="C25">
-        <v>10.039999999999999</v>
+        <v>10.0333265322099</v>
       </c>
       <c r="D25">
         <v>56.463417095520001</v>
@@ -1339,10 +1339,10 @@
         <v>17</v>
       </c>
       <c r="B26">
-        <v>56.402000000000001</v>
+        <v>56.4380259057248</v>
       </c>
       <c r="C26">
-        <v>10.353999999999999</v>
+        <v>10.344737876892401</v>
       </c>
       <c r="D26">
         <v>56.305025691342301</v>
@@ -1359,10 +1359,10 @@
         <v>15</v>
       </c>
       <c r="B27">
-        <v>56.36</v>
+        <v>56.433484774112401</v>
       </c>
       <c r="C27">
-        <v>9.8800000000000008</v>
+        <v>10.054630851767</v>
       </c>
       <c r="D27">
         <v>56.429044475677898</v>
@@ -1379,10 +1379,10 @@
         <v>16</v>
       </c>
       <c r="B28">
-        <v>56.354999999999997</v>
+        <v>56.425347172658597</v>
       </c>
       <c r="C28">
-        <v>10.51</v>
+        <v>10.551672230353001</v>
       </c>
       <c r="D28">
         <v>56.410415033462897</v>
@@ -1419,10 +1419,10 @@
         <v>18</v>
       </c>
       <c r="B30">
-        <v>56.16</v>
+        <v>56.157899397675102</v>
       </c>
       <c r="C30">
-        <v>10.191000000000001</v>
+        <v>10.194004094083001</v>
       </c>
       <c r="D30">
         <v>56.184505349247203</v>
@@ -1439,10 +1439,10 @@
         <v>75</v>
       </c>
       <c r="B31">
-        <v>56.16</v>
+        <v>56.153618307524198</v>
       </c>
       <c r="C31">
-        <v>9.4700000000000006</v>
+        <v>9.5599045517559098</v>
       </c>
       <c r="D31">
         <v>56.150195310444403</v>
@@ -1459,10 +1459,10 @@
         <v>76</v>
       </c>
       <c r="B32">
-        <v>56.16</v>
+        <v>56.161479205457098</v>
       </c>
       <c r="C32">
-        <v>9.5399999999999991</v>
+        <v>9.5586719824484199</v>
       </c>
       <c r="D32">
         <v>56.164895095341301</v>
@@ -1479,10 +1479,10 @@
         <v>77</v>
       </c>
       <c r="B33">
-        <v>56.16</v>
+        <v>56.169894873734499</v>
       </c>
       <c r="C33">
-        <v>9.5399999999999991</v>
+        <v>9.5562490075739408</v>
       </c>
       <c r="D33">
         <v>56.198355159255698</v>
@@ -1539,10 +1539,10 @@
         <v>26</v>
       </c>
       <c r="B36">
-        <v>56.14</v>
+        <v>56.133477154496298</v>
       </c>
       <c r="C36">
-        <v>8.98</v>
+        <v>9.0218845411217501</v>
       </c>
       <c r="D36">
         <v>56.131819052757798</v>
@@ -1559,10 +1559,10 @@
         <v>73</v>
       </c>
       <c r="B37">
-        <v>56.13</v>
+        <v>56.132238694262597</v>
       </c>
       <c r="C37">
-        <v>8.9700000000000006</v>
+        <v>9.0227523536107501</v>
       </c>
       <c r="D37">
         <v>56.120286861733703</v>
@@ -1679,10 +1679,10 @@
         <v>21</v>
       </c>
       <c r="B43">
-        <v>56.034999999999997</v>
+        <v>55.977383849092199</v>
       </c>
       <c r="C43">
-        <v>9.8350000000000009</v>
+        <v>9.8305807611932003</v>
       </c>
       <c r="D43">
         <v>55.972710798681497</v>
@@ -1699,10 +1699,10 @@
         <v>74</v>
       </c>
       <c r="B44">
-        <v>56.03</v>
+        <v>56.052433791569101</v>
       </c>
       <c r="C44">
-        <v>9.85</v>
+        <v>9.7507231015015492</v>
       </c>
       <c r="D44">
         <v>56.147819403046299</v>
@@ -1719,10 +1719,10 @@
         <v>25</v>
       </c>
       <c r="B45">
-        <v>56.026000000000003</v>
+        <v>55.756675042879202</v>
       </c>
       <c r="C45">
-        <v>9.4239999999999995</v>
+        <v>9.4199575363940298</v>
       </c>
       <c r="D45">
         <v>55.718919392443603</v>
@@ -1739,10 +1739,10 @@
         <v>72</v>
       </c>
       <c r="B46">
-        <v>56.02</v>
+        <v>56.186722413267297</v>
       </c>
       <c r="C46">
-        <v>9.3000000000000007</v>
+        <v>9.35171395185629</v>
       </c>
       <c r="D46">
         <v>56.129292344415497</v>
@@ -1759,10 +1759,10 @@
         <v>79</v>
       </c>
       <c r="B47">
-        <v>56</v>
+        <v>56.100441949889998</v>
       </c>
       <c r="C47">
-        <v>8.1199999999999992</v>
+        <v>8.2412990705052405</v>
       </c>
       <c r="D47">
         <v>56.131370778647103</v>
@@ -1779,10 +1779,10 @@
         <v>112</v>
       </c>
       <c r="B48">
-        <v>56</v>
+        <v>56.046333626865703</v>
       </c>
       <c r="C48">
-        <v>12.18</v>
+        <v>12.376769175521799</v>
       </c>
       <c r="D48">
         <v>55.980376482356398</v>
@@ -1799,10 +1799,10 @@
         <v>22</v>
       </c>
       <c r="B49">
-        <v>55.985999999999997</v>
+        <v>55.975680591395196</v>
       </c>
       <c r="C49">
-        <v>9.5120000000000005</v>
+        <v>9.6891890006440402</v>
       </c>
       <c r="D49">
         <v>55.910187302844399</v>
@@ -1819,10 +1819,10 @@
         <v>113</v>
       </c>
       <c r="B50">
-        <v>55.97</v>
+        <v>55.969663052976898</v>
       </c>
       <c r="C50">
-        <v>12.54</v>
+        <v>12.5435350168444</v>
       </c>
       <c r="D50">
         <v>55.9642585158429</v>
@@ -1839,10 +1839,10 @@
         <v>114</v>
       </c>
       <c r="B51">
-        <v>55.97</v>
+        <v>55.927063791968699</v>
       </c>
       <c r="C51">
-        <v>12.5</v>
+        <v>12.511225719199</v>
       </c>
       <c r="D51">
         <v>55.931369747910999</v>
@@ -1859,10 +1859,10 @@
         <v>115</v>
       </c>
       <c r="B52">
-        <v>55.97</v>
+        <v>55.981598803174002</v>
       </c>
       <c r="C52">
-        <v>12.39</v>
+        <v>12.3965742917197</v>
       </c>
       <c r="D52">
         <v>55.902096015783798</v>
@@ -1879,10 +1879,10 @@
         <v>27</v>
       </c>
       <c r="B53">
-        <v>55.935000000000002</v>
+        <v>56.043517384416802</v>
       </c>
       <c r="C53">
-        <v>9.1760000000000002</v>
+        <v>9.05241680521255</v>
       </c>
       <c r="D53">
         <v>56.010817134199897</v>
@@ -1899,10 +1899,10 @@
         <v>108</v>
       </c>
       <c r="B54">
-        <v>55.92</v>
+        <v>55.935097383599199</v>
       </c>
       <c r="C54">
-        <v>12.3</v>
+        <v>12.301733738256701</v>
       </c>
       <c r="D54">
         <v>55.902095883660998</v>
@@ -1919,10 +1919,10 @@
         <v>28</v>
       </c>
       <c r="B55">
-        <v>55.917999999999999</v>
+        <v>55.9197645908745</v>
       </c>
       <c r="C55">
-        <v>9.1449999999999996</v>
+        <v>8.9087351555662497</v>
       </c>
       <c r="D55">
         <v>55.963540247568297</v>
@@ -1939,10 +1939,10 @@
         <v>33</v>
       </c>
       <c r="B56">
-        <v>55.908000000000001</v>
+        <v>55.902734594723199</v>
       </c>
       <c r="C56">
-        <v>9.3780000000000001</v>
+        <v>9.3999548935044306</v>
       </c>
       <c r="D56">
         <v>55.828209896791599</v>
@@ -1959,10 +1959,10 @@
         <v>29</v>
       </c>
       <c r="B57">
-        <v>55.89</v>
+        <v>55.9500180963609</v>
       </c>
       <c r="C57">
-        <v>9.1240000000000006</v>
+        <v>9.1069673229113395</v>
       </c>
       <c r="D57">
         <v>55.943241350166502</v>
@@ -1979,10 +1979,10 @@
         <v>116</v>
       </c>
       <c r="B58">
-        <v>55.88</v>
+        <v>55.883639711821303</v>
       </c>
       <c r="C58">
-        <v>12.53</v>
+        <v>12.544215976369699</v>
       </c>
       <c r="D58">
         <v>55.873587927607197</v>
@@ -1999,10 +1999,10 @@
         <v>23</v>
       </c>
       <c r="B59">
-        <v>55.866999999999997</v>
+        <v>55.874354019834598</v>
       </c>
       <c r="C59">
-        <v>9.907</v>
+        <v>9.8368246922160694</v>
       </c>
       <c r="D59">
         <v>55.882828665757799</v>
@@ -2011,7 +2011,7 @@
         <v>9.7870097765780599</v>
       </c>
       <c r="F59">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2019,10 +2019,10 @@
         <v>117</v>
       </c>
       <c r="B60">
-        <v>55.82</v>
+        <v>55.926155725077699</v>
       </c>
       <c r="C60">
-        <v>12.4</v>
+        <v>12.342060251746799</v>
       </c>
       <c r="D60">
         <v>55.792569263048897</v>
@@ -2039,10 +2039,10 @@
         <v>30</v>
       </c>
       <c r="B61">
-        <v>55.79</v>
+        <v>55.845463865816299</v>
       </c>
       <c r="C61">
-        <v>9.23</v>
+        <v>9.2362145554550708</v>
       </c>
       <c r="D61">
         <v>55.863470581782401</v>
@@ -2059,10 +2059,10 @@
         <v>109</v>
       </c>
       <c r="B62">
-        <v>55.79</v>
+        <v>55.785788161758397</v>
       </c>
       <c r="C62">
-        <v>12.48</v>
+        <v>12.4904981498856</v>
       </c>
       <c r="D62">
         <v>55.779565439616</v>
@@ -2079,10 +2079,10 @@
         <v>61</v>
       </c>
       <c r="B63">
-        <v>55.77</v>
+        <v>55.771191937411103</v>
       </c>
       <c r="C63">
-        <v>11.39</v>
+        <v>11.3917999726538</v>
       </c>
       <c r="D63">
         <v>55.711299630671199</v>
@@ -2099,10 +2099,10 @@
         <v>32</v>
       </c>
       <c r="B64">
-        <v>55.76</v>
+        <v>55.810078304583399</v>
       </c>
       <c r="C64">
-        <v>9.3800000000000008</v>
+        <v>9.3566154016984093</v>
       </c>
       <c r="D64">
         <v>55.8344491603523</v>
@@ -2119,10 +2119,10 @@
         <v>31</v>
       </c>
       <c r="B65">
-        <v>55.735999999999997</v>
+        <v>55.731135192613898</v>
       </c>
       <c r="C65">
-        <v>9.1289999999999996</v>
+        <v>9.1392009249246708</v>
       </c>
       <c r="D65">
         <v>55.839797883900502</v>
@@ -2139,10 +2139,10 @@
         <v>24</v>
       </c>
       <c r="B66">
-        <v>55.707000000000001</v>
+        <v>55.701726587369699</v>
       </c>
       <c r="C66">
-        <v>9.5350000000000001</v>
+        <v>9.4362012684391008</v>
       </c>
       <c r="D66">
         <v>55.748622796829501</v>
@@ -2159,10 +2159,10 @@
         <v>60</v>
       </c>
       <c r="B67">
-        <v>55.698</v>
+        <v>55.693577906559497</v>
       </c>
       <c r="C67">
-        <v>11.77</v>
+        <v>11.7484068284682</v>
       </c>
       <c r="D67">
         <v>55.675403941259198</v>
@@ -2219,10 +2219,10 @@
         <v>56</v>
       </c>
       <c r="B70">
-        <v>55.642000000000003</v>
+        <v>55.642797663225203</v>
       </c>
       <c r="C70">
-        <v>12.083</v>
+        <v>12.0802229001303</v>
       </c>
       <c r="D70">
         <v>55.646679524890899</v>
@@ -2259,10 +2259,10 @@
         <v>59</v>
       </c>
       <c r="B72">
-        <v>55.6</v>
+        <v>55.665478595751203</v>
       </c>
       <c r="C72">
-        <v>11.95</v>
+        <v>12.004401014922401</v>
       </c>
       <c r="D72">
         <v>55.646868298814503</v>
@@ -2279,10 +2279,10 @@
         <v>51</v>
       </c>
       <c r="B73">
-        <v>55.59</v>
+        <v>55.430205513623498</v>
       </c>
       <c r="C73">
-        <v>11.56</v>
+        <v>11.5569077186786</v>
       </c>
       <c r="D73">
         <v>55.458476105181497</v>
@@ -2319,10 +2319,10 @@
         <v>46</v>
       </c>
       <c r="B75">
-        <v>55.58</v>
+        <v>55.569706207844398</v>
       </c>
       <c r="C75">
-        <v>9.7560000000000002</v>
+        <v>9.7572875237505396</v>
       </c>
       <c r="D75">
         <v>55.528470958961499</v>
@@ -2339,10 +2339,10 @@
         <v>58</v>
       </c>
       <c r="B76">
-        <v>55.58</v>
+        <v>55.601355043446702</v>
       </c>
       <c r="C76">
-        <v>11.96</v>
+        <v>11.964859815189699</v>
       </c>
       <c r="D76">
         <v>55.626372502520802</v>
@@ -2359,10 +2359,10 @@
         <v>136</v>
       </c>
       <c r="B77">
-        <v>55.56</v>
+        <v>55.564400011841101</v>
       </c>
       <c r="C77">
-        <v>12.25</v>
+        <v>12.2748413112613</v>
       </c>
       <c r="D77">
         <v>55.579060385517799</v>
@@ -2379,10 +2379,10 @@
         <v>50</v>
       </c>
       <c r="B78">
-        <v>55.53</v>
+        <v>55.510041955016597</v>
       </c>
       <c r="C78">
-        <v>11.39</v>
+        <v>11.378665867076499</v>
       </c>
       <c r="D78">
         <v>55.414777374976197</v>
@@ -2399,10 +2399,10 @@
         <v>91</v>
       </c>
       <c r="B79">
-        <v>55.517000000000003</v>
+        <v>55.418011763554901</v>
       </c>
       <c r="C79">
-        <v>9.5050000000000008</v>
+        <v>9.5673791591495299</v>
       </c>
       <c r="D79">
         <v>55.434860149355302</v>
@@ -2439,10 +2439,10 @@
         <v>45</v>
       </c>
       <c r="B81">
-        <v>55.509</v>
+        <v>55.507933356480798</v>
       </c>
       <c r="C81">
-        <v>9.7309999999999999</v>
+        <v>9.7197213852796107</v>
       </c>
       <c r="D81">
         <v>55.510939959172603</v>
@@ -2459,10 +2459,10 @@
         <v>54</v>
       </c>
       <c r="B82">
-        <v>55.5</v>
+        <v>55.465215042151598</v>
       </c>
       <c r="C82">
-        <v>12</v>
+        <v>12.120388349372201</v>
       </c>
       <c r="D82">
         <v>55.467939971445603</v>
@@ -2479,10 +2479,10 @@
         <v>89</v>
       </c>
       <c r="B83">
-        <v>55.497999999999998</v>
+        <v>55.4999953261906</v>
       </c>
       <c r="C83">
-        <v>9.5839999999999996</v>
+        <v>9.5323465498743296</v>
       </c>
       <c r="D83">
         <v>55.537262434396297</v>
@@ -2499,10 +2499,10 @@
         <v>140</v>
       </c>
       <c r="B84">
-        <v>55.49</v>
+        <v>55.566698506107798</v>
       </c>
       <c r="C84">
-        <v>9.74</v>
+        <v>9.7586806821170597</v>
       </c>
       <c r="D84">
         <v>55.471148161042301</v>
@@ -2519,10 +2519,10 @@
         <v>90</v>
       </c>
       <c r="B85">
-        <v>55.484000000000002</v>
+        <v>55.491741936143001</v>
       </c>
       <c r="C85">
-        <v>9.4749999999999996</v>
+        <v>9.4747937400949294</v>
       </c>
       <c r="D85">
         <v>55.462567395252698</v>
@@ -2599,10 +2599,10 @@
         <v>87</v>
       </c>
       <c r="B89">
-        <v>55.46</v>
+        <v>55.451860537563697</v>
       </c>
       <c r="C89">
-        <v>9.11</v>
+        <v>9.0382764112568594</v>
       </c>
       <c r="D89">
         <v>55.503697666734602</v>
@@ -2619,10 +2619,10 @@
         <v>52</v>
       </c>
       <c r="B90">
-        <v>55.45</v>
+        <v>55.445617104884597</v>
       </c>
       <c r="C90">
-        <v>11.75</v>
+        <v>11.7874313670739</v>
       </c>
       <c r="D90">
         <v>55.456868094755499</v>
@@ -2639,10 +2639,10 @@
         <v>86</v>
       </c>
       <c r="B91">
-        <v>55.44</v>
+        <v>55.410356333543596</v>
       </c>
       <c r="C91">
-        <v>9.07</v>
+        <v>8.96650606521691</v>
       </c>
       <c r="D91">
         <v>55.521807028186998</v>
@@ -2659,10 +2659,10 @@
         <v>49</v>
       </c>
       <c r="B92">
-        <v>55.433999999999997</v>
+        <v>55.3496595734659</v>
       </c>
       <c r="C92">
-        <v>11.458</v>
+        <v>11.5047984852733</v>
       </c>
       <c r="D92">
         <v>55.388308639384398</v>
@@ -2679,10 +2679,10 @@
         <v>35</v>
       </c>
       <c r="B93">
-        <v>55.433</v>
+        <v>55.443551770409499</v>
       </c>
       <c r="C93">
-        <v>10.635</v>
+        <v>10.617701603333201</v>
       </c>
       <c r="D93">
         <v>55.352277207549903</v>
@@ -2699,10 +2699,10 @@
         <v>36</v>
       </c>
       <c r="B94">
-        <v>55.42</v>
+        <v>55.353028661191402</v>
       </c>
       <c r="C94">
-        <v>10.53</v>
+        <v>10.532064468071701</v>
       </c>
       <c r="D94">
         <v>55.352277207549903</v>
@@ -2719,10 +2719,10 @@
         <v>48</v>
       </c>
       <c r="B95">
-        <v>55.405000000000001</v>
+        <v>55.394753042122403</v>
       </c>
       <c r="C95">
-        <v>11.378</v>
+        <v>11.272486251725899</v>
       </c>
       <c r="D95">
         <v>55.366080534430999</v>
@@ -2739,10 +2739,10 @@
         <v>38</v>
       </c>
       <c r="B96">
-        <v>55.398000000000003</v>
+        <v>55.398619115870098</v>
       </c>
       <c r="C96">
-        <v>10.387</v>
+        <v>10.3918586298115</v>
       </c>
       <c r="D96">
         <v>55.348040950998502</v>
@@ -2759,10 +2759,10 @@
         <v>42</v>
       </c>
       <c r="B97">
-        <v>55.393999999999998</v>
+        <v>55.396088109913102</v>
       </c>
       <c r="C97">
-        <v>10.38</v>
+        <v>10.3813911554372</v>
       </c>
       <c r="D97">
         <v>55.386245803765398</v>
@@ -2779,10 +2779,10 @@
         <v>41</v>
       </c>
       <c r="B98">
-        <v>55.393000000000001</v>
+        <v>55.402823810375203</v>
       </c>
       <c r="C98">
-        <v>10.384</v>
+        <v>10.3870508112549</v>
       </c>
       <c r="D98">
         <v>55.359155061782502</v>
@@ -2799,10 +2799,10 @@
         <v>37</v>
       </c>
       <c r="B99">
-        <v>55.384999999999998</v>
+        <v>55.420136757003498</v>
       </c>
       <c r="C99">
-        <v>10.334</v>
+        <v>10.362427746660501</v>
       </c>
       <c r="D99">
         <v>55.365572638557701</v>
@@ -2819,10 +2819,10 @@
         <v>39</v>
       </c>
       <c r="B100">
-        <v>55.378</v>
+        <v>55.378732071426697</v>
       </c>
       <c r="C100">
-        <v>10.37</v>
+        <v>10.371917138234799</v>
       </c>
       <c r="D100">
         <v>55.352084838587601</v>
@@ -2839,10 +2839,10 @@
         <v>43</v>
       </c>
       <c r="B101">
-        <v>55.37</v>
+        <v>55.383437870124503</v>
       </c>
       <c r="C101">
-        <v>10.15</v>
+        <v>10.1307976191775</v>
       </c>
       <c r="D101">
         <v>55.398716088410197</v>
@@ -2859,10 +2859,10 @@
         <v>40</v>
       </c>
       <c r="B102">
-        <v>55.362000000000002</v>
+        <v>55.366674119237999</v>
       </c>
       <c r="C102">
-        <v>10.37</v>
+        <v>10.3858889265996</v>
       </c>
       <c r="D102">
         <v>55.352084838587601</v>
@@ -2879,10 +2879,10 @@
         <v>92</v>
       </c>
       <c r="B103">
-        <v>55.34</v>
+        <v>55.356620247797402</v>
       </c>
       <c r="C103">
-        <v>9.4700000000000006</v>
+        <v>9.4866313586135007</v>
       </c>
       <c r="D103">
         <v>55.366860664522299</v>
@@ -2899,10 +2899,10 @@
         <v>47</v>
       </c>
       <c r="B104">
-        <v>55.337000000000003</v>
+        <v>55.3339734275052</v>
       </c>
       <c r="C104">
-        <v>11.138999999999999</v>
+        <v>11.137360270780899</v>
       </c>
       <c r="D104">
         <v>55.354211586724198</v>
@@ -2939,10 +2939,10 @@
         <v>85</v>
       </c>
       <c r="B106">
-        <v>55.32</v>
+        <v>55.326944919993601</v>
       </c>
       <c r="C106">
-        <v>8.76</v>
+        <v>8.7741222730983193</v>
       </c>
       <c r="D106">
         <v>55.521807028186998</v>
@@ -2959,10 +2959,10 @@
         <v>34</v>
       </c>
       <c r="B107">
-        <v>55.308999999999997</v>
+        <v>55.3127764993095</v>
       </c>
       <c r="C107">
-        <v>10.792999999999999</v>
+        <v>10.787373884270499</v>
       </c>
       <c r="D107">
         <v>55.305637430336603</v>
@@ -2979,10 +2979,10 @@
         <v>84</v>
       </c>
       <c r="B108">
-        <v>55.295000000000002</v>
+        <v>55.295832839957001</v>
       </c>
       <c r="C108">
-        <v>8.657</v>
+        <v>8.6694189131063908</v>
       </c>
       <c r="D108">
         <v>55.505653111481898</v>
@@ -3039,10 +3039,10 @@
         <v>119</v>
       </c>
       <c r="B111">
-        <v>55.25</v>
+        <v>55.286762948353001</v>
       </c>
       <c r="C111">
-        <v>11.83</v>
+        <v>11.815719628452101</v>
       </c>
       <c r="D111">
         <v>55.344885143290298</v>
@@ -3099,10 +3099,10 @@
         <v>94</v>
       </c>
       <c r="B114">
-        <v>55.22</v>
+        <v>55.237902297283803</v>
       </c>
       <c r="C114">
-        <v>9.57</v>
+        <v>9.3737696572867204</v>
       </c>
       <c r="D114">
         <v>55.250630030225899</v>
@@ -3119,10 +3119,10 @@
         <v>104</v>
       </c>
       <c r="B115">
-        <v>55.19</v>
+        <v>55.176369648190303</v>
       </c>
       <c r="C115">
-        <v>10.47</v>
+        <v>10.4907326652077</v>
       </c>
       <c r="D115">
         <v>55.194239428249901</v>
@@ -3139,10 +3139,10 @@
         <v>123</v>
       </c>
       <c r="B116">
-        <v>55.19</v>
+        <v>55.218580235913599</v>
       </c>
       <c r="C116">
-        <v>11.79</v>
+        <v>11.796271130305101</v>
       </c>
       <c r="D116">
         <v>55.173291438901899</v>
@@ -3159,10 +3159,10 @@
         <v>122</v>
       </c>
       <c r="B117">
-        <v>55.16</v>
+        <v>55.1894322152786</v>
       </c>
       <c r="C117">
-        <v>11.75</v>
+        <v>11.7223663829255</v>
       </c>
       <c r="D117">
         <v>55.173291438901899</v>
@@ -3179,10 +3179,10 @@
         <v>124</v>
       </c>
       <c r="B118">
-        <v>55.12</v>
+        <v>55.175662996272798</v>
       </c>
       <c r="C118">
-        <v>12.08</v>
+        <v>12.098651599347299</v>
       </c>
       <c r="D118">
         <v>55.079583894118997</v>
@@ -3199,10 +3199,10 @@
         <v>102</v>
       </c>
       <c r="B119">
-        <v>55.1</v>
+        <v>55.127069819649101</v>
       </c>
       <c r="C119">
-        <v>10.199999999999999</v>
+        <v>10.2551127037618</v>
       </c>
       <c r="D119">
         <v>55.311469148101303</v>
@@ -3219,10 +3219,10 @@
         <v>95</v>
       </c>
       <c r="B120">
-        <v>55.08</v>
+        <v>55.134917600540902</v>
       </c>
       <c r="C120">
-        <v>9.48</v>
+        <v>9.4437445378350997</v>
       </c>
       <c r="D120">
         <v>55.177860208956197</v>
@@ -3239,10 +3239,10 @@
         <v>105</v>
       </c>
       <c r="B121">
-        <v>55.06</v>
+        <v>55.063888144855703</v>
       </c>
       <c r="C121">
-        <v>10.64</v>
+        <v>10.6076541652033</v>
       </c>
       <c r="D121">
         <v>55.119567952856698</v>
@@ -3259,10 +3259,10 @@
         <v>99</v>
       </c>
       <c r="B122">
-        <v>55.05</v>
+        <v>54.903045346267199</v>
       </c>
       <c r="C122">
-        <v>9.74</v>
+        <v>9.7486066437832495</v>
       </c>
       <c r="D122">
         <v>54.9261740861104</v>
@@ -3299,10 +3299,10 @@
         <v>96</v>
       </c>
       <c r="B124">
-        <v>55.04</v>
+        <v>55.0394998144616</v>
       </c>
       <c r="C124">
-        <v>9.41</v>
+        <v>9.4145374400771793</v>
       </c>
       <c r="D124">
         <v>54.988018952115397</v>
@@ -3319,10 +3319,10 @@
         <v>98</v>
       </c>
       <c r="B125">
-        <v>55.04</v>
+        <v>54.906935761982098</v>
       </c>
       <c r="C125">
-        <v>9.7899999999999991</v>
+        <v>9.7831609006020592</v>
       </c>
       <c r="D125">
         <v>54.920897557935398</v>
@@ -3339,10 +3339,10 @@
         <v>106</v>
       </c>
       <c r="B126">
-        <v>55.04</v>
+        <v>55.059635343286502</v>
       </c>
       <c r="C126">
-        <v>10.61</v>
+        <v>10.614773212815599</v>
       </c>
       <c r="D126">
         <v>55.0774328705401</v>
@@ -3359,10 +3359,10 @@
         <v>125</v>
       </c>
       <c r="B127">
-        <v>55</v>
+        <v>55.007391352173201</v>
       </c>
       <c r="C127">
-        <v>11.9</v>
+        <v>11.9131682707681</v>
       </c>
       <c r="D127">
         <v>55.0065379793555</v>
@@ -3379,10 +3379,10 @@
         <v>107</v>
       </c>
       <c r="B128">
-        <v>54.99</v>
+        <v>55.0224636793671</v>
       </c>
       <c r="C128">
-        <v>10.69</v>
+        <v>10.6537546400764</v>
       </c>
       <c r="D128">
         <v>55.063145900389799</v>
@@ -3399,10 +3399,10 @@
         <v>126</v>
       </c>
       <c r="B129">
-        <v>54.96</v>
+        <v>54.965630652450599</v>
       </c>
       <c r="C129">
-        <v>12.54</v>
+        <v>12.5462719218778</v>
       </c>
       <c r="D129">
         <v>54.9557618106438</v>
@@ -3419,10 +3419,10 @@
         <v>101</v>
       </c>
       <c r="B130">
-        <v>54.93</v>
+        <v>54.928538268149602</v>
       </c>
       <c r="C130">
-        <v>9.8699999999999992</v>
+        <v>9.5963147786884093</v>
       </c>
       <c r="D130">
         <v>54.952232890230597</v>
@@ -3479,10 +3479,10 @@
         <v>97</v>
       </c>
       <c r="B133">
-        <v>54.83</v>
+        <v>54.844297937771699</v>
       </c>
       <c r="C133">
-        <v>9.27</v>
+        <v>9.3277812400695694</v>
       </c>
       <c r="D133">
         <v>54.863456153378301</v>
@@ -3539,10 +3539,10 @@
         <v>129</v>
       </c>
       <c r="B136">
-        <v>54.78</v>
+        <v>54.775191572896603</v>
       </c>
       <c r="C136">
-        <v>11.88</v>
+        <v>11.8407041754717</v>
       </c>
       <c r="D136">
         <v>54.828311504111298</v>
@@ -3559,10 +3559,10 @@
         <v>134</v>
       </c>
       <c r="B137">
-        <v>54.78</v>
+        <v>54.704914493668802</v>
       </c>
       <c r="C137">
-        <v>11.33</v>
+        <v>11.4017951977763</v>
       </c>
       <c r="D137">
         <v>54.665534941541402</v>
@@ -3579,10 +3579,10 @@
         <v>130</v>
       </c>
       <c r="B138">
-        <v>54.77</v>
+        <v>54.723975986486799</v>
       </c>
       <c r="C138">
-        <v>11.81</v>
+        <v>11.799988492170799</v>
       </c>
       <c r="D138">
         <v>54.795000494061902</v>

</xml_diff>